<commit_message>
kind of finished with the generator, still fo fix the total cost missing and nan errore in corsi
</commit_message>
<xml_diff>
--- a/V5/problemGenerator/timetablingTemplate.xlsx
+++ b/V5/problemGenerator/timetablingTemplate.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="corsi" sheetId="1" state="visible" r:id="rId3"/>
@@ -13,6 +13,7 @@
     <sheet name="disponibilitàProfessori" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="disponibilitàAule" sheetId="4" state="visible" r:id="rId6"/>
     <sheet name="disponibilitàScdla" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="configurazione" sheetId="6" state="visible" r:id="rId8"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -24,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="80">
   <si>
     <t xml:space="preserve">corso</t>
   </si>
@@ -243,16 +244,38 @@
   </si>
   <si>
     <t xml:space="preserve">scdla</t>
+  </si>
+  <si>
+    <t xml:space="preserve">configurazioni</t>
+  </si>
+  <si>
+    <t xml:space="preserve">valori</t>
+  </si>
+  <si>
+    <t xml:space="preserve">orario a costo minimo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DA IMPLEMENTARE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">orario nel quale inserire un ora di pausa pranzo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">valorizzare il tenere le giornate vuote?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">valorizzare il tenere le mezze giornate vuote?</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="General"/>
+    <numFmt numFmtId="165" formatCode="General"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -274,6 +297,18 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -318,12 +353,20 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2040,7 +2083,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:BD3"/>
+  <dimension ref="A1:BD10"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2551,6 +2594,242 @@
       </c>
       <c r="BD3" s="1" t="n">
         <v>1</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="F4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="I4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="J4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="K4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="L4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="M4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="N4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="O4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="P4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="R4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="S4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="T4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="U4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="V4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="W4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="X4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AK4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AL4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AM4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AO4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AP4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AS4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AV4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AW4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AZ4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="BA4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="BB4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="BC4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="BD4" s="1" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G10" s="2" t="n">
+        <f aca="false">configurazione!B3</f>
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Normale"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Normale"&amp;12&amp;KffffffPagina &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:C5"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40.52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="18.26"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="0" t="s">
+        <v>73</v>
+      </c>
+      <c r="B1" s="0" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="0" t="s">
+        <v>75</v>
+      </c>
+      <c r="B2" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="C2" s="0" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="0" t="s">
+        <v>77</v>
+      </c>
+      <c r="B3" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="0" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="3" t="s">
+        <v>79</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fixed total cost missing and nan errore in corsi, still ti implement a lot of things
</commit_message>
<xml_diff>
--- a/V5/problemGenerator/timetablingTemplate.xlsx
+++ b/V5/problemGenerator/timetablingTemplate.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="5"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="corsi" sheetId="1" state="visible" r:id="rId3"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="80">
   <si>
     <t xml:space="preserve">corso</t>
   </si>
@@ -271,9 +271,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
-    <numFmt numFmtId="165" formatCode="General"/>
   </numFmts>
   <fonts count="6">
     <font>
@@ -362,7 +361,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2597,180 +2596,65 @@
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C4" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D4" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="E4" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="F4" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="G4" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="H4" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="I4" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="J4" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="K4" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="L4" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="M4" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="N4" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="O4" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="P4" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q4" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="R4" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="S4" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="T4" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="U4" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="V4" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="W4" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="X4" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="Y4" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="Z4" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="AA4" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="AB4" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC4" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="AD4" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="AE4" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="AF4" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="AG4" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="AH4" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="AI4" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="AJ4" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="AK4" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="AL4" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="AM4" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="AN4" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="AO4" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="AP4" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="AQ4" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="AR4" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="AS4" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="AT4" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="AU4" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="AV4" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="AW4" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="AX4" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="AY4" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="AZ4" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="BA4" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="BB4" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="BC4" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="BD4" s="1" t="n">
-        <v>1</v>
-      </c>
+      <c r="A4" s="1"/>
+      <c r="B4" s="1"/>
+      <c r="C4" s="1"/>
+      <c r="D4" s="1"/>
+      <c r="E4" s="1"/>
+      <c r="F4" s="1"/>
+      <c r="G4" s="1"/>
+      <c r="H4" s="1"/>
+      <c r="I4" s="1"/>
+      <c r="J4" s="1"/>
+      <c r="K4" s="1"/>
+      <c r="L4" s="1"/>
+      <c r="M4" s="1"/>
+      <c r="N4" s="1"/>
+      <c r="O4" s="1"/>
+      <c r="P4" s="1"/>
+      <c r="Q4" s="1"/>
+      <c r="R4" s="1"/>
+      <c r="S4" s="1"/>
+      <c r="T4" s="1"/>
+      <c r="U4" s="1"/>
+      <c r="V4" s="1"/>
+      <c r="W4" s="1"/>
+      <c r="X4" s="1"/>
+      <c r="Y4" s="1"/>
+      <c r="Z4" s="1"/>
+      <c r="AA4" s="1"/>
+      <c r="AB4" s="1"/>
+      <c r="AC4" s="1"/>
+      <c r="AD4" s="1"/>
+      <c r="AE4" s="1"/>
+      <c r="AF4" s="1"/>
+      <c r="AG4" s="1"/>
+      <c r="AH4" s="1"/>
+      <c r="AI4" s="1"/>
+      <c r="AJ4" s="1"/>
+      <c r="AK4" s="1"/>
+      <c r="AL4" s="1"/>
+      <c r="AM4" s="1"/>
+      <c r="AN4" s="1"/>
+      <c r="AO4" s="1"/>
+      <c r="AP4" s="1"/>
+      <c r="AQ4" s="1"/>
+      <c r="AR4" s="1"/>
+      <c r="AS4" s="1"/>
+      <c r="AT4" s="1"/>
+      <c r="AU4" s="1"/>
+      <c r="AV4" s="1"/>
+      <c r="AW4" s="1"/>
+      <c r="AX4" s="1"/>
+      <c r="AY4" s="1"/>
+      <c r="AZ4" s="1"/>
+      <c r="BA4" s="1"/>
+      <c r="BB4" s="1"/>
+      <c r="BC4" s="1"/>
+      <c r="BD4" s="1"/>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G10" s="2" t="n">
-        <f aca="false">configurazione!B3</f>
-        <v>0</v>
-      </c>
+      <c r="G10" s="2"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>